<commit_message>
Atualiza fotos da equipe
</commit_message>
<xml_diff>
--- a/_input_data/tsiino_hiiwiida_team.xlsx
+++ b/_input_data/tsiino_hiiwiida_team.xlsx
@@ -11,7 +11,7 @@
     <sheet name="team" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">team!$A$1:$I$79</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">team!$A$1:$I$78</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="304">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -1489,7 +1489,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P1004"/>
+  <dimension ref="A1:P1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.36"/>
@@ -1589,115 +1589,123 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="6" t="s">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
+      <c r="I6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="H7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="2" t="s">
-        <v>31</v>
+      <c r="G8" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="7" t="s">
-        <v>38</v>
+      <c r="G9" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>10</v>
@@ -1708,21 +1716,23 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>48</v>
+      </c>
       <c r="G10" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>10</v>
@@ -1733,118 +1743,116 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>46</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>48</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>56</v>
+      </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="G12" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I12" s="2"/>
+      <c r="I12" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>58</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="E14" s="2"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="G14" s="2"/>
       <c r="H14" s="2" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="G15" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="H15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1854,146 +1862,144 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="2" t="s">
-        <v>75</v>
-      </c>
+      <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="G17" s="2"/>
       <c r="H17" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>78</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="E18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>85</v>
+      </c>
       <c r="H18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I18" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>85</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
       <c r="H19" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>87</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
+        <v>92</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I20" s="9"/>
+      <c r="I20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+        <v>93</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="G21" s="7" t="s">
+        <v>96</v>
+      </c>
       <c r="H21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I21" s="2"/>
+      <c r="I21" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>95</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="7" t="s">
-        <v>96</v>
+      <c r="G22" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>10</v>
@@ -2004,331 +2010,333 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="G23" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>10</v>
+        <v>106</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>110</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>110</v>
+        <v>115</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>116</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>116</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D27" s="2"/>
+      <c r="A27" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="10"/>
       <c r="E27" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
+      </c>
+      <c r="F27" s="10"/>
+      <c r="G27" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I27" s="2"/>
+      <c r="I27" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="D28" s="10"/>
-      <c r="E28" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F28" s="10"/>
-      <c r="G28" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="H28" s="2" t="s">
+      <c r="A28" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I28" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="H29" s="6" t="s">
+      <c r="A29" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I29" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
+      <c r="I29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B30" s="2"/>
+        <v>136</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>137</v>
+      </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="E30" s="2" t="s">
+        <v>138</v>
+      </c>
       <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="G30" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="H30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I30" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>141</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>86</v>
+        <v>145</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>142</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="2" t="s">
-        <v>143</v>
-      </c>
+      <c r="E32" s="2"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="2" t="s">
-        <v>144</v>
-      </c>
+      <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>146</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2" t="s">
+      <c r="A33" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D33" s="10"/>
+      <c r="E33" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" s="10"/>
-      <c r="E34" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
+      <c r="I34" s="2" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>152</v>
+        <v>55</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D36" s="2"/>
-      <c r="E36" s="2" t="s">
-        <v>158</v>
+      <c r="E36" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="F36" s="2"/>
-      <c r="G36" s="2" t="s">
-        <v>159</v>
+      <c r="G36" s="7" t="s">
+        <v>163</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>10</v>
@@ -2339,92 +2347,90 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>161</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="2"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="11" t="s">
-        <v>162</v>
-      </c>
+      <c r="E37" s="11"/>
       <c r="F37" s="2"/>
-      <c r="G37" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="G37" s="7"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>35</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="11"/>
+      <c r="E38" s="2"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="I38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>167</v>
+      </c>
       <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="E39" s="2" t="s">
+        <v>168</v>
+      </c>
       <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+      <c r="G39" s="2" t="s">
+        <v>169</v>
+      </c>
       <c r="H39" s="2" t="s">
-        <v>10</v>
+        <v>170</v>
       </c>
       <c r="I39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>61</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="B40" s="2"/>
       <c r="C40" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D40" s="2"/>
-      <c r="E40" s="2" t="s">
-        <v>168</v>
-      </c>
+      <c r="E40" s="2"/>
       <c r="F40" s="2"/>
-      <c r="G40" s="2" t="s">
-        <v>169</v>
-      </c>
+      <c r="G40" s="2"/>
       <c r="H40" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="I40" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B41" s="2"/>
+        <v>173</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="C41" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
+      <c r="E41" s="2" t="s">
+        <v>175</v>
+      </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2" t="s">
@@ -2436,42 +2442,42 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D42" s="2"/>
-      <c r="E42" s="2" t="s">
-        <v>175</v>
-      </c>
+      <c r="E42" s="2"/>
       <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
+      <c r="G42" s="2" t="s">
+        <v>178</v>
+      </c>
       <c r="H42" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I42" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>61</v>
+        <v>180</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
+      <c r="E43" s="2" t="s">
+        <v>182</v>
+      </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>10</v>
@@ -2480,118 +2486,110 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D44" s="2"/>
-      <c r="E44" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2" t="s">
-        <v>183</v>
+      <c r="E44" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>189</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I44" s="2"/>
+      <c r="I44" s="2" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>186</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
       <c r="D45" s="2"/>
-      <c r="E45" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>189</v>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>87</v>
-      </c>
+      <c r="I45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B46" s="2"/>
+        <v>192</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>193</v>
+      </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="H47" s="2" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="D47" s="9"/>
+      <c r="E47" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="F47" s="9"/>
+      <c r="G47" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="H47" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="D48" s="9"/>
-      <c r="E48" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="F48" s="9"/>
-      <c r="G48" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="H48" s="9" t="s">
+      <c r="I47" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I48" s="9" t="s">
-        <v>17</v>
-      </c>
+      <c r="I48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -2606,7 +2604,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -2621,139 +2619,143 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
+        <v>202</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>203</v>
+      </c>
       <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
+      <c r="E51" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>206</v>
+      </c>
       <c r="H51" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I51" s="2"/>
+      <c r="I51" s="2" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>61</v>
+        <v>209</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D52" s="2"/>
+        <v>210</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>211</v>
+      </c>
       <c r="E52" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F52" s="11" t="s">
-        <v>205</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>206</v>
+        <v>212</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>214</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>207</v>
+        <v>146</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>209</v>
+        <v>40</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>211</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="D53" s="2"/>
       <c r="E53" s="2" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>146</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>40</v>
+        <v>221</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D54" s="2"/>
+        <v>222</v>
+      </c>
+      <c r="D54" s="9"/>
       <c r="E54" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F54" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>219</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
       <c r="H54" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I54" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="D55" s="9"/>
+        <v>225</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
       <c r="E55" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="F55" s="9"/>
-      <c r="G55" s="9"/>
+        <v>226</v>
+      </c>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2" t="s">
+        <v>227</v>
+      </c>
       <c r="H55" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I55" s="9"/>
+      <c r="I55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C56" s="2"/>
+        <v>229</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>230</v>
+      </c>
       <c r="D56" s="2"/>
-      <c r="E56" s="2" t="s">
-        <v>226</v>
-      </c>
+      <c r="E56" s="2"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="2" t="s">
-        <v>227</v>
-      </c>
+      <c r="G56" s="2"/>
       <c r="H56" s="2" t="s">
         <v>10</v>
       </c>
@@ -2761,16 +2763,18 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>229</v>
+        <v>61</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
+      <c r="E57" s="2" t="s">
+        <v>233</v>
+      </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2" t="s">
@@ -2780,20 +2784,22 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
+      <c r="G58" s="2" t="s">
+        <v>237</v>
+      </c>
       <c r="H58" s="2" t="s">
         <v>10</v>
       </c>
@@ -2801,63 +2807,59 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>61</v>
+        <v>239</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F59" s="2"/>
+        <v>241</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>242</v>
+      </c>
       <c r="G59" s="2" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I59" s="2"/>
+        <v>244</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>240</v>
-      </c>
+        <v>246</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>243</v>
-      </c>
+        <v>247</v>
+      </c>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
       <c r="H60" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>245</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I60" s="2"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="B61" s="2"/>
+        <v>248</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>249</v>
+      </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
@@ -2868,16 +2870,12 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>249</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
-      <c r="E62" s="2" t="s">
-        <v>250</v>
-      </c>
+      <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2" t="s">
@@ -2887,7 +2885,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -2902,10 +2900,14 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
+        <v>253</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
@@ -2913,47 +2915,49 @@
       <c r="H64" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I64" s="2"/>
+      <c r="I64" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>45</v>
+        <v>239</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
+      <c r="E65" s="2" t="s">
+        <v>257</v>
+      </c>
       <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
+      <c r="G65" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="H65" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I65" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I65" s="2"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="F66" s="2"/>
-      <c r="G66" s="2" t="s">
-        <v>258</v>
-      </c>
+      <c r="G66" s="2"/>
       <c r="H66" s="2" t="s">
         <v>10</v>
       </c>
@@ -2961,17 +2965,17 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>260</v>
+        <v>35</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
@@ -2982,78 +2986,78 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>264</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
       <c r="D68" s="2"/>
-      <c r="E68" s="2" t="s">
-        <v>265</v>
-      </c>
+      <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I68" s="2"/>
+      <c r="I68" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
+        <v>267</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>270</v>
+      </c>
       <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
+      <c r="F69" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>272</v>
+      </c>
       <c r="H69" s="2" t="s">
-        <v>10</v>
+        <v>273</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>17</v>
+        <v>274</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>270</v>
-      </c>
-      <c r="E70" s="2"/>
-      <c r="F70" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>272</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="F70" s="2"/>
+      <c r="G70" s="2"/>
       <c r="H70" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>274</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I70" s="2"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
+        <v>277</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>279</v>
+      </c>
       <c r="D71" s="2"/>
       <c r="E71" s="2" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
@@ -3064,20 +3068,16 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>279</v>
-      </c>
+        <v>281</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
       <c r="D72" s="2"/>
-      <c r="E72" s="2" t="s">
-        <v>280</v>
-      </c>
+      <c r="E72" s="2"/>
       <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
+      <c r="G72" s="2" t="s">
+        <v>282</v>
+      </c>
       <c r="H72" s="2" t="s">
         <v>10</v>
       </c>
@@ -3085,16 +3085,20 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
+        <v>283</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>284</v>
+      </c>
       <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
+      <c r="E73" s="2" t="s">
+        <v>285</v>
+      </c>
       <c r="F73" s="2"/>
-      <c r="G73" s="2" t="s">
-        <v>282</v>
-      </c>
+      <c r="G73" s="2"/>
       <c r="H73" s="2" t="s">
         <v>10</v>
       </c>
@@ -3102,18 +3106,12 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>284</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
       <c r="D74" s="2"/>
-      <c r="E74" s="2" t="s">
-        <v>285</v>
-      </c>
+      <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2" t="s">
@@ -3123,121 +3121,117 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
+        <v>287</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>288</v>
+      </c>
       <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
+      <c r="E75" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="F75" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>291</v>
+      </c>
       <c r="H75" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I75" s="2"/>
+      <c r="I75" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>288</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="C76" s="2"/>
       <c r="D76" s="2"/>
-      <c r="E76" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="F76" s="8" t="s">
-        <v>290</v>
-      </c>
+      <c r="E76" s="2"/>
+      <c r="F76" s="2"/>
       <c r="G76" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I76" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="I76" s="2"/>
+      <c r="J76" s="13"/>
+      <c r="K76" s="13"/>
+      <c r="L76" s="13"/>
+      <c r="M76" s="13"/>
+      <c r="N76" s="13"/>
+      <c r="O76" s="13"/>
+      <c r="P76" s="13"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C77" s="2"/>
+        <v>295</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>296</v>
+      </c>
       <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
+      <c r="E77" s="2" t="s">
+        <v>297</v>
+      </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I77" s="2"/>
-      <c r="J77" s="13"/>
-      <c r="K77" s="13"/>
-      <c r="L77" s="13"/>
-      <c r="M77" s="13"/>
-      <c r="N77" s="13"/>
-      <c r="O77" s="13"/>
-      <c r="P77" s="13"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2" t="s">
-        <v>294</v>
+      <c r="A78" s="14" t="s">
+        <v>299</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>295</v>
+        <v>14</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D78" s="2"/>
-      <c r="E78" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="F78" s="2"/>
+      <c r="E78" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="F78" s="10" t="s">
+        <v>302</v>
+      </c>
       <c r="G78" s="2" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I78" s="2"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="14" t="s">
-        <v>299</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="D79" s="2"/>
-      <c r="E79" s="10" t="s">
-        <v>301</v>
-      </c>
-      <c r="F79" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="H79" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I79" s="2" t="s">
+      <c r="I78" s="2" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="79" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="9"/>
+      <c r="B79" s="9"/>
+      <c r="C79" s="9"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9"/>
+      <c r="G79" s="9"/>
+      <c r="H79" s="9"/>
+      <c r="I79" s="9"/>
     </row>
     <row r="80" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="9"/>
@@ -13403,52 +13397,42 @@
       <c r="H1003" s="9"/>
       <c r="I1003" s="9"/>
     </row>
-    <row r="1004" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1004" s="9"/>
-      <c r="B1004" s="9"/>
-      <c r="C1004" s="9"/>
-      <c r="D1004" s="9"/>
-      <c r="E1004" s="9"/>
-      <c r="F1004" s="9"/>
-      <c r="G1004" s="9"/>
-      <c r="H1004" s="9"/>
-      <c r="I1004" s="9"/>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:I79"/>
+  <autoFilter ref="A1:I78"/>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" display="https://www.instagram.com/anaflabio?igsh=ZXpqZnZ6djhvZnQ4"/>
-    <hyperlink ref="E6" r:id="rId2" display="https://lattes.cnpq.br/0954834722824284"/>
-    <hyperlink ref="G6" r:id="rId3" display="https://orcid.org/0000-0002-5641-024X"/>
-    <hyperlink ref="G9" r:id="rId4" display="https://orcid.org/0009-0008-3121-7436"/>
-    <hyperlink ref="F11" r:id="rId5" display="https://scholar.google.com.br/citations?user=rlWY7rQAAAAJ&amp;hl=pt-PT"/>
-    <hyperlink ref="F13" r:id="rId6" display="https://scholar.google.es/citations?hl=en&amp;user=6C8ozYwAAAAJ"/>
-    <hyperlink ref="F19" r:id="rId7" display="https://scholar.google.com.br/citations?user=yyOMVXIAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G19" r:id="rId8" display="https://orcid.org/0000-0002-5081-2803"/>
-    <hyperlink ref="E20" r:id="rId9" display="http://lattes.cnpq.br/4816888485402257"/>
-    <hyperlink ref="G22" r:id="rId10" display="https://orcid.org/0000-0001-6623-3788"/>
-    <hyperlink ref="F25" r:id="rId11" display="https://scholar.google.com/citations?user=QC55kc8AAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="E28" r:id="rId12" display="http://lattes.cnpq.br/3062370237651162"/>
-    <hyperlink ref="D29" r:id="rId13" display="https://www.instagram.com/bonesfabio/"/>
-    <hyperlink ref="E29" r:id="rId14" display="https://lattes.cnpq.br/7058195011982806"/>
-    <hyperlink ref="F29" r:id="rId15" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G29" r:id="rId16" display="https://orcid.org/0000-0003-2956-1859"/>
-    <hyperlink ref="E34" r:id="rId17" display="http://lattes.cnpq.br/3177536756466033"/>
-    <hyperlink ref="E37" r:id="rId18" display="http://lattes.cnpq.br/4435352680317467"/>
-    <hyperlink ref="G37" r:id="rId19" display="https://orcid.org/0009-0000-5487-0915"/>
-    <hyperlink ref="E45" r:id="rId20" display="http://lattes.cnpq.br/6183123558330376"/>
-    <hyperlink ref="F45" r:id="rId21" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G45" r:id="rId22" display="https://orcid.org/0000-0002-3193-9315"/>
-    <hyperlink ref="E48" r:id="rId23" display="http://lattes.cnpq.br/8595257513343424"/>
-    <hyperlink ref="G48" r:id="rId24" display="https://orcid.org/0000-0002-9696-1978"/>
-    <hyperlink ref="F52" r:id="rId25" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G52" r:id="rId26" display="https://orcid.org/0000-0001-8441-2106 "/>
-    <hyperlink ref="D53" r:id="rId27" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
-    <hyperlink ref="F53" r:id="rId28" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="F54" r:id="rId29" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
-    <hyperlink ref="D70" r:id="rId30" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
-    <hyperlink ref="F70" r:id="rId31" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
-    <hyperlink ref="F76" r:id="rId32" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D5" r:id="rId1" display="https://www.instagram.com/anaflabio?igsh=ZXpqZnZ6djhvZnQ4"/>
+    <hyperlink ref="E5" r:id="rId2" display="https://lattes.cnpq.br/0954834722824284"/>
+    <hyperlink ref="G5" r:id="rId3" display="https://orcid.org/0000-0002-5641-024X"/>
+    <hyperlink ref="G8" r:id="rId4" display="https://orcid.org/0009-0008-3121-7436"/>
+    <hyperlink ref="F10" r:id="rId5" display="https://scholar.google.com.br/citations?user=rlWY7rQAAAAJ&amp;hl=pt-PT"/>
+    <hyperlink ref="F12" r:id="rId6" display="https://scholar.google.es/citations?hl=en&amp;user=6C8ozYwAAAAJ"/>
+    <hyperlink ref="F18" r:id="rId7" display="https://scholar.google.com.br/citations?user=yyOMVXIAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G18" r:id="rId8" display="https://orcid.org/0000-0002-5081-2803"/>
+    <hyperlink ref="E19" r:id="rId9" display="http://lattes.cnpq.br/4816888485402257"/>
+    <hyperlink ref="G21" r:id="rId10" display="https://orcid.org/0000-0001-6623-3788"/>
+    <hyperlink ref="F24" r:id="rId11" display="https://scholar.google.com/citations?user=QC55kc8AAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="E27" r:id="rId12" display="http://lattes.cnpq.br/3062370237651162"/>
+    <hyperlink ref="D28" r:id="rId13" display="https://www.instagram.com/bonesfabio/"/>
+    <hyperlink ref="E28" r:id="rId14" display="https://lattes.cnpq.br/7058195011982806"/>
+    <hyperlink ref="F28" r:id="rId15" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G28" r:id="rId16" display="https://orcid.org/0000-0003-2956-1859"/>
+    <hyperlink ref="E33" r:id="rId17" display="http://lattes.cnpq.br/3177536756466033"/>
+    <hyperlink ref="E36" r:id="rId18" display="http://lattes.cnpq.br/4435352680317467"/>
+    <hyperlink ref="G36" r:id="rId19" display="https://orcid.org/0009-0000-5487-0915"/>
+    <hyperlink ref="E44" r:id="rId20" display="http://lattes.cnpq.br/6183123558330376"/>
+    <hyperlink ref="F44" r:id="rId21" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G44" r:id="rId22" display="https://orcid.org/0000-0002-3193-9315"/>
+    <hyperlink ref="E47" r:id="rId23" display="http://lattes.cnpq.br/8595257513343424"/>
+    <hyperlink ref="G47" r:id="rId24" display="https://orcid.org/0000-0002-9696-1978"/>
+    <hyperlink ref="F51" r:id="rId25" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G51" r:id="rId26" display="https://orcid.org/0000-0001-8441-2106 "/>
+    <hyperlink ref="D52" r:id="rId27" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
+    <hyperlink ref="F52" r:id="rId28" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="F53" r:id="rId29" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D69" r:id="rId30" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
+    <hyperlink ref="F69" r:id="rId31" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
+    <hyperlink ref="F75" r:id="rId32" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Adiciona validador de planilha de herbario e atualiza site
</commit_message>
<xml_diff>
--- a/_input_data/tsiino_hiiwiida_team.xlsx
+++ b/_input_data/tsiino_hiiwiida_team.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="320">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -307,9 +307,35 @@
     <t xml:space="preserve">https://scholar.google.com/citations?user=dGyQqDEAAAAJ&amp;hl=pt-BR&amp;oi=ao</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://orcid.org/0000-0002-8851-0202
+</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Dayana Martins Rodrigues</t>
   </si>
   <si>
+    <t xml:space="preserve">UFAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dayanamartins501@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.instagram.com/dayrodrigues978?igsh=MXh5bjN6ZXIxYXdvNg==</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2669986623645624</t>
+  </si>
+  <si>
     <t xml:space="preserve">Débora Zuanny</t>
   </si>
   <si>
@@ -604,6 +630,21 @@
     <t xml:space="preserve">Jo Wilbraham</t>
   </si>
   <si>
+    <t xml:space="preserve">NHM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j.wilbraham@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/jo-wilbraham.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
     <t xml:space="preserve">https://orcid.org/0000-0003-4101-0611</t>
   </si>
   <si>
@@ -634,6 +675,12 @@
     <t xml:space="preserve">Jovita Yesilyurt</t>
   </si>
   <si>
+    <t xml:space="preserve">j.yesilyurt@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kleuto Moraes da Silva</t>
   </si>
   <si>
@@ -778,9 +825,6 @@
     <t xml:space="preserve">Nelcioney José de Souza Araújo</t>
   </si>
   <si>
-    <t xml:space="preserve">UFAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">http://lattes.cnpq.br/5403024203206579</t>
   </si>
   <si>
@@ -875,6 +919,15 @@
   </si>
   <si>
     <t xml:space="preserve">Silvia Pressel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.pressel@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/silvia-pressel.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en</t>
   </si>
   <si>
     <t xml:space="preserve">https://orcid.org/0000-0001-9652-6338</t>
@@ -950,7 +1003,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1035,6 +1088,14 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -1131,7 +1192,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1177,6 +1238,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1189,6 +1258,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1939,7 +2012,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="31" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>89</v>
       </c>
@@ -1956,41 +2029,58 @@
       <c r="F19" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="11" t="s">
+        <v>94</v>
+      </c>
       <c r="H19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3" t="s">
+      <c r="A20" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I20" s="3"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>10</v>
@@ -2001,19 +2091,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>10</v>
@@ -2024,26 +2114,26 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>88</v>
@@ -2051,26 +2141,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>61</v>
@@ -2078,26 +2168,26 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>17</v>
@@ -2105,21 +2195,21 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>10</v>
@@ -2127,22 +2217,22 @@
       <c r="I26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="B27" s="11" t="s">
+      <c r="A27" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D27" s="11"/>
+      <c r="C27" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" s="14"/>
       <c r="E27" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" s="11"/>
+        <v>133</v>
+      </c>
+      <c r="F27" s="14"/>
       <c r="G27" s="10" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>10</v>
@@ -2153,31 +2243,31 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>10</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
@@ -2189,7 +2279,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2204,19 +2294,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>87</v>
@@ -2227,32 +2317,32 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2266,18 +2356,18 @@
       <c r="I32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="B33" s="11" t="s">
+      <c r="A33" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C33" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="D33" s="11"/>
+      <c r="C33" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="D33" s="14"/>
       <c r="E33" s="3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -2286,21 +2376,21 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>10</v>
@@ -2311,21 +2401,21 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>10</v>
@@ -2336,21 +2426,21 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D36" s="3"/>
-      <c r="E36" s="12" t="s">
-        <v>164</v>
+      <c r="E36" s="15" t="s">
+        <v>169</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="8" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>10</v>
@@ -2361,14 +2451,14 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B37" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B37" s="14" t="s">
         <v>35</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="12"/>
+      <c r="E37" s="15"/>
       <c r="F37" s="3"/>
       <c r="G37" s="8"/>
       <c r="H37" s="3"/>
@@ -2376,7 +2466,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2391,34 +2481,34 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="I39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
@@ -2433,17 +2523,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -2456,19 +2546,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>10</v>
@@ -2477,21 +2567,21 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>10</v>
@@ -2500,23 +2590,23 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>10</v>
@@ -2526,35 +2616,52 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="H45" s="3" t="s">
+      <c r="A45" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="G45" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="H45" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I45" s="3"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="13"/>
+      <c r="K45" s="13"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="13"/>
+      <c r="N45" s="13"/>
+      <c r="O45" s="13"/>
+      <c r="P45" s="13"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>10</v>
@@ -2563,21 +2670,21 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="D47" s="10"/>
-      <c r="E47" s="13" t="s">
-        <v>199</v>
+      <c r="E47" s="16" t="s">
+        <v>209</v>
       </c>
       <c r="F47" s="10"/>
-      <c r="G47" s="13" t="s">
-        <v>200</v>
+      <c r="G47" s="16" t="s">
+        <v>210</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>10</v>
@@ -2588,7 +2695,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2602,23 +2709,36 @@
       <c r="I48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3" t="s">
+      <c r="A49" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I49" s="3"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="13"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="13"/>
+      <c r="N49" s="13"/>
+      <c r="O49" s="13"/>
+      <c r="P49" s="13"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2633,79 +2753,79 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>207</v>
+        <v>218</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>219</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>10</v>
@@ -2716,17 +2836,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="3" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
@@ -2737,19 +2857,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>10</v>
@@ -2758,13 +2878,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -2777,17 +2897,17 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -2798,21 +2918,21 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>10</v>
@@ -2821,40 +2941,40 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -2865,15 +2985,15 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>251</v>
+        <v>96</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -2884,7 +3004,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -2899,7 +3019,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -2914,13 +3034,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -2935,21 +3055,21 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="D65" s="3"/>
       <c r="E65" s="3" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>10</v>
@@ -2958,17 +3078,17 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -2979,17 +3099,17 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="3" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -3000,7 +3120,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -3017,40 +3137,40 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="9" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -3061,17 +3181,17 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="3" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -3081,35 +3201,52 @@
       <c r="I71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="H72" s="3" t="s">
+      <c r="A72" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="B72" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="E72" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="G72" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="H72" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I72" s="3"/>
+      <c r="I72" s="13"/>
+      <c r="J72" s="13"/>
+      <c r="K72" s="13"/>
+      <c r="L72" s="13"/>
+      <c r="M72" s="13"/>
+      <c r="N72" s="13"/>
+      <c r="O72" s="13"/>
+      <c r="P72" s="13"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -3120,7 +3257,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -3135,23 +3272,23 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="D75" s="3"/>
       <c r="E75" s="3" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>10</v>
@@ -3162,7 +3299,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>61</v>
@@ -3172,37 +3309,37 @@
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
       <c r="G76" s="3" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I76" s="3"/>
-      <c r="J76" s="14"/>
-      <c r="K76" s="14"/>
-      <c r="L76" s="14"/>
-      <c r="M76" s="14"/>
-      <c r="N76" s="14"/>
-      <c r="O76" s="14"/>
-      <c r="P76" s="14"/>
+      <c r="J76" s="17"/>
+      <c r="K76" s="17"/>
+      <c r="L76" s="17"/>
+      <c r="M76" s="17"/>
+      <c r="N76" s="17"/>
+      <c r="O76" s="17"/>
+      <c r="P76" s="17"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="3" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>10</v>
@@ -3210,24 +3347,24 @@
       <c r="I77" s="3"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="15" t="s">
-        <v>301</v>
+      <c r="A78" s="18" t="s">
+        <v>315</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="D78" s="3"/>
-      <c r="E78" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="F78" s="11" t="s">
-        <v>304</v>
+      <c r="E78" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="F78" s="14" t="s">
+        <v>318</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>10</v>
@@ -13424,29 +13561,37 @@
     <hyperlink ref="F18" r:id="rId7" display="https://scholar.google.com.br/citations?user=yyOMVXIAAAAJ&amp;hl=pt-BR"/>
     <hyperlink ref="G18" r:id="rId8" display="https://orcid.org/0000-0002-5081-2803"/>
     <hyperlink ref="E19" r:id="rId9" display="http://lattes.cnpq.br/4816888485402257"/>
-    <hyperlink ref="G21" r:id="rId10" display="https://orcid.org/0000-0001-6623-3788"/>
-    <hyperlink ref="F24" r:id="rId11" display="https://scholar.google.com/citations?user=QC55kc8AAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="E27" r:id="rId12" display="http://lattes.cnpq.br/3062370237651162"/>
-    <hyperlink ref="D28" r:id="rId13" display="https://www.instagram.com/bonesfabio/"/>
-    <hyperlink ref="E28" r:id="rId14" display="https://lattes.cnpq.br/7058195011982806"/>
-    <hyperlink ref="F28" r:id="rId15" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G28" r:id="rId16" display="https://orcid.org/0000-0003-2956-1859"/>
-    <hyperlink ref="E33" r:id="rId17" display="http://lattes.cnpq.br/3177536756466033"/>
-    <hyperlink ref="E36" r:id="rId18" display="http://lattes.cnpq.br/4435352680317467"/>
-    <hyperlink ref="G36" r:id="rId19" display="https://orcid.org/0009-0000-5487-0915"/>
-    <hyperlink ref="E44" r:id="rId20" display="http://lattes.cnpq.br/6183123558330376"/>
-    <hyperlink ref="F44" r:id="rId21" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G44" r:id="rId22" display="https://orcid.org/0000-0002-3193-9315"/>
-    <hyperlink ref="E47" r:id="rId23" display="http://lattes.cnpq.br/8595257513343424"/>
-    <hyperlink ref="G47" r:id="rId24" display="https://orcid.org/0000-0002-9696-1978"/>
-    <hyperlink ref="F51" r:id="rId25" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G51" r:id="rId26" display="https://orcid.org/0000-0001-8441-2106 "/>
-    <hyperlink ref="D52" r:id="rId27" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
-    <hyperlink ref="F52" r:id="rId28" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="F53" r:id="rId29" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
-    <hyperlink ref="D69" r:id="rId30" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
-    <hyperlink ref="F69" r:id="rId31" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
-    <hyperlink ref="F75" r:id="rId32" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D20" r:id="rId10" display="https://www.instagram.com/dayrodrigues978?igsh=MXh5bjN6ZXIxYXdvNg=="/>
+    <hyperlink ref="E20" r:id="rId11" display="http://lattes.cnpq.br/2669986623645624"/>
+    <hyperlink ref="G21" r:id="rId12" display="https://orcid.org/0000-0001-6623-3788"/>
+    <hyperlink ref="F24" r:id="rId13" display="https://scholar.google.com/citations?user=QC55kc8AAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="E27" r:id="rId14" display="http://lattes.cnpq.br/3062370237651162"/>
+    <hyperlink ref="D28" r:id="rId15" display="https://www.instagram.com/bonesfabio/"/>
+    <hyperlink ref="E28" r:id="rId16" display="https://lattes.cnpq.br/7058195011982806"/>
+    <hyperlink ref="F28" r:id="rId17" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G28" r:id="rId18" display="https://orcid.org/0000-0003-2956-1859"/>
+    <hyperlink ref="E33" r:id="rId19" display="http://lattes.cnpq.br/3177536756466033"/>
+    <hyperlink ref="E36" r:id="rId20" display="http://lattes.cnpq.br/4435352680317467"/>
+    <hyperlink ref="G36" r:id="rId21" display="https://orcid.org/0009-0000-5487-0915"/>
+    <hyperlink ref="E44" r:id="rId22" display="http://lattes.cnpq.br/6183123558330376"/>
+    <hyperlink ref="F44" r:id="rId23" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G44" r:id="rId24" display="https://orcid.org/0000-0002-3193-9315"/>
+    <hyperlink ref="D45" r:id="rId25" display="https://www.nhm.ac.uk/our-science/people/jo-wilbraham.html"/>
+    <hyperlink ref="G45" r:id="rId26" display="https://orcid.org/0000-0003-4101-0611"/>
+    <hyperlink ref="E47" r:id="rId27" display="http://lattes.cnpq.br/8595257513343424"/>
+    <hyperlink ref="G47" r:id="rId28" display="https://orcid.org/0000-0002-9696-1978"/>
+    <hyperlink ref="D49" r:id="rId29" display="https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html"/>
+    <hyperlink ref="F51" r:id="rId30" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G51" r:id="rId31" display="https://orcid.org/0000-0001-8441-2106 "/>
+    <hyperlink ref="D52" r:id="rId32" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
+    <hyperlink ref="F52" r:id="rId33" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="F53" r:id="rId34" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D69" r:id="rId35" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
+    <hyperlink ref="F69" r:id="rId36" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
+    <hyperlink ref="D72" r:id="rId37" display="https://www.nhm.ac.uk/our-science/people/silvia-pressel.html"/>
+    <hyperlink ref="F72" r:id="rId38" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
+    <hyperlink ref="G72" r:id="rId39" display="https://orcid.org/0000-0001-9652-6338"/>
+    <hyperlink ref="F75" r:id="rId40" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13455,6 +13600,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId33"/>
+  <drawing r:id="rId41"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza validador de herbário e dados do site
</commit_message>
<xml_diff>
--- a/_input_data/tsiino_hiiwiida_team.xlsx
+++ b/_input_data/tsiino_hiiwiida_team.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="325">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -307,18 +307,8 @@
     <t xml:space="preserve">https://scholar.google.com/citations?user=dGyQqDEAAAAJ&amp;hl=pt-BR&amp;oi=ao</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://orcid.org/0000-0002-8851-0202
+    <t xml:space="preserve">https://orcid.org/0000-0002-8851-0202
 </t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Dayana Martins Rodrigues</t>
@@ -642,358 +632,373 @@
     <t xml:space="preserve">n/a</t>
   </si>
   <si>
+    <t xml:space="preserve">https://orcid.org/0000-0003-4101-0611</t>
+  </si>
+  <si>
+    <t xml:space="preserve">João Paulo Machado de Araújo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural History Museum of Denmark/University of Copenhagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0003-2529-7691</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jone C R Mendes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jonecmendes5@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/8595257513343424</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-9696-1978</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Roberto Pinho de Andrade Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jovita Yesilyurt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j.yesilyurt@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kleuto Moraes da Silva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layon O. Demarchi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">layon.lod@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2504309339279053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-8441-2106 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAPEAM/CNPq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leandro Giacomin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UFPB/PPG-Bot INPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">giacomin.leandro@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/1944885983694994</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-8862-4042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luciano Paganucci de Queiroz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luciano.paganucci@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/0424535851535945</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-7436-0939</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luísa Azevedo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural History Museum, Londres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luisaazevedomeyer@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/4997896034406339</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luiz Henrique Vieira Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UFRPE/PGS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lattes.cnpq.br/8928747588815635</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-7623-2826</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcus Vinicius Gonçalves da Silva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvinicius.gsilva2003@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maria de Lourdes da Costa Soares Morais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soares@inpa.gov.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/9125127898290625</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael John Gilbert Hopkins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mikehopkins44@hotmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/7971117717977278</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-5473-2942</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micheline Carvalho-Silva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UnB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">silvamicheline@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/1015868478480965</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?hl=en&amp;user=_xgrCh0AAAAJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-2389-3804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pesquisadora responsável FAPDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAPDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moisés Luiz da Silva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2995553227548402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nelcioney José de Souza Araújo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/5403024203206579</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ocírio de Souza Pereira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onalto Ferreira de Menezes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paolo de Castro Martins Massoni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paolo.massoni@jbrj.gov.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paulo Eduardo Aguiar Saraiva Câmara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paducamara@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2742831544064073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-3944-996X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedro Lage Viana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pedro.viana@inma.gov.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/8375441896375273</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rafaela Saraiva Peres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rafaelasaraiva82@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/8803152023599223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renato Vieira Soares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandra Diane Knapp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural History Museum, London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.knapp@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/sandra-knapp.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-7698-3945</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-lead; Pesquisadora responsável UKRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UKRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selma Lúcia de Moura Gonzales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/5473538959324771</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shirley Cunha Feuerstein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shirley.feuerstein@ifto.edu.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/5697367502174932</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silvia Pressel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s.pressel@nhm.ac.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/silvia-pressel.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0001-9652-6338</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tales Alves Júnior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tjfilho01@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/8055018980718354</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiago de Medeiros Mouzinho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuane Bochorny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tbochorny@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2127883418769406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0003-1953-8516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiara Sousa Cabral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0003-0187-3498</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valdely Ferreira Kinupp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFAM Campus Manaus-Zona Leste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">val@ifam.edu.br</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/1263334983122560</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-3892-7288</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valner Jordão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valner.jordao@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/5405013641413074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://scholar.google.com/citations?user=sWg8vA0AAAAJ&amp;hl=pt-BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-6328-0738</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleissa de Oliveira Martins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cleissab.i.o@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.instagram.com/cleissa_oliveira99/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/5162929358710284</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">https://orcid.org/0000-0003-4101-0611</t>
-  </si>
-  <si>
-    <t xml:space="preserve">João Paulo Machado de Araújo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natural History Museum of Denmark/University of Copenhagen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0003-2529-7691</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jone C R Mendes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jonecmendes5@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/8595257513343424</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-9696-1978</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Roberto Pinho de Andrade Lima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jovita Yesilyurt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">j.yesilyurt@nhm.ac.uk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kleuto Moraes da Silva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Layon O. Demarchi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">layon.lod@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/2504309339279053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-8441-2106 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAPEAM/CNPq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leandro Giacomin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UFPB/PPG-Bot INPA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">giacomin.leandro@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/1944885983694994</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-8862-4042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luciano Paganucci de Queiroz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">luciano.paganucci@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/0424535851535945</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-7436-0939</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luísa Azevedo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natural History Museum, Londres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">luisaazevedomeyer@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/4997896034406339</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luiz Henrique Vieira Lima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UFRPE/PGS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lattes.cnpq.br/8928747588815635</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-7623-2826</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marcus Vinicius Gonçalves da Silva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mvinicius.gsilva2003@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maria de Lourdes da Costa Soares Morais</t>
-  </si>
-  <si>
-    <t xml:space="preserve">soares@inpa.gov.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/9125127898290625</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michael John Gilbert Hopkins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mikehopkins44@hotmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/7971117717977278</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-5473-2942</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Micheline Carvalho-Silva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UnB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">silvamicheline@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/1015868478480965</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?hl=en&amp;user=_xgrCh0AAAAJ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-2389-3804</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pesquisadora responsável FAPDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAPDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moisés Luiz da Silva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/2995553227548402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nelcioney José de Souza Araújo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/5403024203206579</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ocírio de Souza Pereira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onalto Ferreira de Menezes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paolo de Castro Martins Massoni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paolo.massoni@jbrj.gov.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paulo Eduardo Aguiar Saraiva Câmara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paducamara@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/2742831544064073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-3944-996X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pedro Lage Viana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pedro.viana@inma.gov.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/8375441896375273</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rafaela Saraiva Peres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rafaelasaraiva82@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/8803152023599223</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renato Vieira Soares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandra Diane Knapp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natural History Museum, London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s.knapp@nhm.ac.uk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/sandra-knapp.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-7698-3945</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-lead; Pesquisadora responsável UKRI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UKRI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selma Lúcia de Moura Gonzales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/5473538959324771</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shirley Cunha Feuerstein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">shirley.feuerstein@ifto.edu.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/5697367502174932</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silvia Pressel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s.pressel@nhm.ac.uk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.nhm.ac.uk/our-science/people/silvia-pressel.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-9652-6338</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tales Alves Júnior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tjfilho01@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/8055018980718354</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiago de Medeiros Mouzinho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thuane Bochorny</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tbochorny@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/2127883418769406</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0003-1953-8516</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiara Sousa Cabral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0003-0187-3498</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valdely Ferreira Kinupp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFAM Campus Manaus-Zona Leste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">val@ifam.edu.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/1263334983122560</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-3892-7288</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valner Jordão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valner.jordao@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://lattes.cnpq.br/5405013641413074</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://scholar.google.com/citations?user=sWg8vA0AAAAJ&amp;hl=pt-BR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-6328-0738</t>
+    <t xml:space="preserve">https://orcid.org/0009-0006-0651-3028</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1197,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1241,11 +1246,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1266,6 +1271,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1403,31 +1416,31 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="e97132"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196b24"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="a02b93"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4ea72e"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
@@ -2012,7 +2025,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="31" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="56" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>89</v>
       </c>
@@ -2631,11 +2644,9 @@
       <c r="E45" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="F45" s="13" t="s">
+      <c r="F45" s="13"/>
+      <c r="G45" s="12" t="s">
         <v>202</v>
-      </c>
-      <c r="G45" s="12" t="s">
-        <v>203</v>
       </c>
       <c r="H45" s="12" t="s">
         <v>10</v>
@@ -2651,17 +2662,17 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>10</v>
@@ -2670,21 +2681,21 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D47" s="10"/>
       <c r="E47" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>10</v>
@@ -2695,7 +2706,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2710,16 +2721,16 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>198</v>
       </c>
       <c r="C49" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D49" s="12" t="s">
         <v>213</v>
-      </c>
-      <c r="D49" s="12" t="s">
-        <v>214</v>
       </c>
       <c r="E49" s="13"/>
       <c r="F49" s="13"/>
@@ -2738,7 +2749,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2753,52 +2764,52 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F51" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="F51" s="15" t="s">
+      <c r="G51" s="8" t="s">
         <v>219</v>
-      </c>
-      <c r="G51" s="8" t="s">
-        <v>220</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="C52" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="D52" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="E52" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="F52" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="F52" s="8" t="s">
+      <c r="G52" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>10</v>
@@ -2809,23 +2820,23 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="F53" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="F53" s="8" t="s">
+      <c r="G53" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>233</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>10</v>
@@ -2836,17 +2847,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B54" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="C54" s="3" t="s">
         <v>235</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>236</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
@@ -2857,19 +2868,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>239</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>10</v>
@@ -2878,13 +2889,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B56" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="C56" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -2897,17 +2908,17 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -2918,21 +2929,21 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>10</v>
@@ -2941,40 +2952,40 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="C59" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>254</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="G59" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="G59" s="3" t="s">
+      <c r="H59" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="H59" s="3" t="s">
+      <c r="I59" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -2985,7 +2996,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>96</v>
@@ -2993,7 +3004,7 @@
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -3004,7 +3015,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -3019,7 +3030,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -3034,13 +3045,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -3055,21 +3066,21 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>269</v>
       </c>
       <c r="D65" s="3"/>
       <c r="E65" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>10</v>
@@ -3078,17 +3089,17 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B66" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="C66" s="3" t="s">
         <v>273</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>274</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -3099,17 +3110,17 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -3120,7 +3131,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -3137,40 +3148,40 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B69" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="C69" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="D69" s="9" t="s">
         <v>282</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>283</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="G69" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="G69" s="3" t="s">
+      <c r="H69" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="H69" s="3" t="s">
+      <c r="I69" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -3181,17 +3192,17 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="C71" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>292</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -3202,25 +3213,25 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B72" s="12" t="s">
         <v>198</v>
       </c>
       <c r="C72" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D72" s="12" t="s">
         <v>295</v>
-      </c>
-      <c r="D72" s="12" t="s">
-        <v>296</v>
       </c>
       <c r="E72" s="12" t="s">
         <v>201</v>
       </c>
       <c r="F72" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="G72" s="12" t="s">
         <v>297</v>
-      </c>
-      <c r="G72" s="12" t="s">
-        <v>298</v>
       </c>
       <c r="H72" s="12" t="s">
         <v>10</v>
@@ -3236,17 +3247,17 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -3257,7 +3268,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -3272,23 +3283,23 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D75" s="3"/>
       <c r="E75" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="F75" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="G75" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>10</v>
@@ -3299,7 +3310,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>61</v>
@@ -3309,7 +3320,7 @@
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
       <c r="G76" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>10</v>
@@ -3325,21 +3336,21 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="B77" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>312</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>10</v>
@@ -3348,23 +3359,23 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="18" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="F78" s="14" t="s">
         <v>317</v>
       </c>
-      <c r="F78" s="14" t="s">
+      <c r="G78" s="3" t="s">
         <v>318</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>319</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>10</v>
@@ -3373,16 +3384,39 @@
         <v>17</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="10"/>
-      <c r="B79" s="10"/>
-      <c r="C79" s="10"/>
-      <c r="D79" s="10"/>
-      <c r="E79" s="10"/>
-      <c r="F79" s="10"/>
-      <c r="G79" s="10"/>
-      <c r="H79" s="10"/>
-      <c r="I79" s="10"/>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="B79" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C79" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="D79" s="19" t="s">
+        <v>321</v>
+      </c>
+      <c r="E79" s="19" t="s">
+        <v>322</v>
+      </c>
+      <c r="F79" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="G79" s="19" t="s">
+        <v>324</v>
+      </c>
+      <c r="H79" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I79" s="20"/>
+      <c r="J79" s="20"/>
+      <c r="K79" s="20"/>
+      <c r="L79" s="20"/>
+      <c r="M79" s="20"/>
+      <c r="N79" s="20"/>
+      <c r="O79" s="20"/>
+      <c r="P79" s="20"/>
     </row>
     <row r="80" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10"/>
@@ -13592,6 +13626,9 @@
     <hyperlink ref="F72" r:id="rId38" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
     <hyperlink ref="G72" r:id="rId39" display="https://orcid.org/0000-0001-9652-6338"/>
     <hyperlink ref="F75" r:id="rId40" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D79" r:id="rId41" display="https://www.instagram.com/cleissa_oliveira99/"/>
+    <hyperlink ref="E79" r:id="rId42" display="http://lattes.cnpq.br/5162929358710284"/>
+    <hyperlink ref="G79" r:id="rId43" display="https://orcid.org/0009-0006-0651-3028"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13600,6 +13637,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId41"/>
+  <drawing r:id="rId44"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
atualizar fotos da equipe
</commit_message>
<xml_diff>
--- a/_input_data/tsiino_hiiwiida_team.xlsx
+++ b/_input_data/tsiino_hiiwiida_team.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="328">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -413,9 +413,15 @@
     <t xml:space="preserve">egross@uesc.br</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.uesc.br/centros/cme/index.php?item=conteudo_equipe.php</t>
+  </si>
+  <si>
     <t xml:space="preserve">http://lattes.cnpq.br/2078633938003826</t>
   </si>
   <si>
+    <t xml:space="preserve">https://scholar.google.com.br/citations?user=11C9o4sAAAAJ&amp;hl=pt-PT</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://orcid.org/0000-0002-1057-0432</t>
   </si>
   <si>
@@ -995,10 +1001,13 @@
     <t xml:space="preserve">http://lattes.cnpq.br/5162929358710284</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
     <t xml:space="preserve">https://orcid.org/0009-0006-0651-3028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alice Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allicelima29@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1197,7 +1206,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1271,14 +1280,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2207,45 +2208,58 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3" t="s">
+      <c r="D26" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3" t="s">
+      <c r="E26" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="F26" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="H26" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I26" s="3"/>
+      <c r="I26" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F27" s="14"/>
       <c r="G27" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>10</v>
@@ -2256,31 +2270,31 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>10</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
@@ -2292,7 +2306,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2307,19 +2321,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>87</v>
@@ -2330,32 +2344,32 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2370,17 +2384,17 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>35</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
@@ -2389,21 +2403,21 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>10</v>
@@ -2414,21 +2428,21 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>10</v>
@@ -2439,21 +2453,21 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="15" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>10</v>
@@ -2464,7 +2478,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>35</v>
@@ -2479,7 +2493,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2494,34 +2508,34 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
@@ -2536,17 +2550,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -2559,19 +2573,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>10</v>
@@ -2580,21 +2594,21 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>10</v>
@@ -2603,23 +2617,23 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>10</v>
@@ -2630,23 +2644,23 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F45" s="13"/>
       <c r="G45" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H45" s="12" t="s">
         <v>10</v>
@@ -2662,17 +2676,17 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>10</v>
@@ -2681,21 +2695,21 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>45</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D47" s="10"/>
       <c r="E47" s="16" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="16" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H47" s="10" t="s">
         <v>10</v>
@@ -2706,7 +2720,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2721,16 +2735,16 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E49" s="13"/>
       <c r="F49" s="13"/>
@@ -2749,7 +2763,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2764,79 +2778,79 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F51" s="15" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>10</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>10</v>
@@ -2847,17 +2861,17 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
@@ -2868,19 +2882,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>10</v>
@@ -2889,13 +2903,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -2908,17 +2922,17 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -2929,21 +2943,21 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>10</v>
@@ -2952,40 +2966,40 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -2996,7 +3010,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>96</v>
@@ -3004,7 +3018,7 @@
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -3015,7 +3029,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -3030,7 +3044,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -3045,13 +3059,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -3066,21 +3080,21 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D65" s="3"/>
       <c r="E65" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>10</v>
@@ -3089,17 +3103,17 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -3110,17 +3124,17 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -3131,7 +3145,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -3148,40 +3162,40 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -3192,17 +3206,17 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -3213,25 +3227,25 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E72" s="12" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F72" s="12" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H72" s="12" t="s">
         <v>10</v>
@@ -3247,17 +3261,17 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -3268,7 +3282,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -3283,23 +3297,23 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D75" s="3"/>
       <c r="E75" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>10</v>
@@ -3310,7 +3324,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>61</v>
@@ -3320,7 +3334,7 @@
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
       <c r="G76" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>10</v>
@@ -3336,21 +3350,21 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>10</v>
@@ -3359,23 +3373,23 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="18" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" s="14" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F78" s="14" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>10</v>
@@ -3385,49 +3399,62 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="19" t="s">
-        <v>319</v>
-      </c>
-      <c r="B79" s="19" t="s">
+      <c r="A79" s="12" t="s">
+        <v>321</v>
+      </c>
+      <c r="B79" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C79" s="19" t="s">
-        <v>320</v>
-      </c>
-      <c r="D79" s="19" t="s">
-        <v>321</v>
-      </c>
-      <c r="E79" s="19" t="s">
+      <c r="C79" s="12" t="s">
         <v>322</v>
       </c>
-      <c r="F79" s="20" t="s">
+      <c r="D79" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="G79" s="19" t="s">
+      <c r="E79" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="H79" s="19" t="s">
+      <c r="F79" s="13"/>
+      <c r="G79" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="H79" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="I79" s="20"/>
-      <c r="J79" s="20"/>
-      <c r="K79" s="20"/>
-      <c r="L79" s="20"/>
-      <c r="M79" s="20"/>
-      <c r="N79" s="20"/>
-      <c r="O79" s="20"/>
-      <c r="P79" s="20"/>
-    </row>
-    <row r="80" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="10"/>
-      <c r="B80" s="10"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-      <c r="E80" s="10"/>
-      <c r="F80" s="10"/>
-      <c r="G80" s="10"/>
-      <c r="H80" s="10"/>
-      <c r="I80" s="10"/>
+      <c r="I79" s="13"/>
+      <c r="J79" s="13"/>
+      <c r="K79" s="13"/>
+      <c r="L79" s="13"/>
+      <c r="M79" s="13"/>
+      <c r="N79" s="13"/>
+      <c r="O79" s="13"/>
+      <c r="P79" s="13"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="B80" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="D80" s="13"/>
+      <c r="E80" s="13"/>
+      <c r="F80" s="13"/>
+      <c r="G80" s="13"/>
+      <c r="H80" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="I80" s="13"/>
+      <c r="J80" s="13"/>
+      <c r="K80" s="13"/>
+      <c r="L80" s="13"/>
+      <c r="M80" s="13"/>
+      <c r="N80" s="13"/>
+      <c r="O80" s="13"/>
+      <c r="P80" s="13"/>
     </row>
     <row r="81" customFormat="false" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
@@ -13599,36 +13626,40 @@
     <hyperlink ref="E20" r:id="rId11" display="http://lattes.cnpq.br/2669986623645624"/>
     <hyperlink ref="G21" r:id="rId12" display="https://orcid.org/0000-0001-6623-3788"/>
     <hyperlink ref="F24" r:id="rId13" display="https://scholar.google.com/citations?user=QC55kc8AAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="E27" r:id="rId14" display="http://lattes.cnpq.br/3062370237651162"/>
-    <hyperlink ref="D28" r:id="rId15" display="https://www.instagram.com/bonesfabio/"/>
-    <hyperlink ref="E28" r:id="rId16" display="https://lattes.cnpq.br/7058195011982806"/>
-    <hyperlink ref="F28" r:id="rId17" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G28" r:id="rId18" display="https://orcid.org/0000-0003-2956-1859"/>
-    <hyperlink ref="E33" r:id="rId19" display="http://lattes.cnpq.br/3177536756466033"/>
-    <hyperlink ref="E36" r:id="rId20" display="http://lattes.cnpq.br/4435352680317467"/>
-    <hyperlink ref="G36" r:id="rId21" display="https://orcid.org/0009-0000-5487-0915"/>
-    <hyperlink ref="E44" r:id="rId22" display="http://lattes.cnpq.br/6183123558330376"/>
-    <hyperlink ref="F44" r:id="rId23" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G44" r:id="rId24" display="https://orcid.org/0000-0002-3193-9315"/>
-    <hyperlink ref="D45" r:id="rId25" display="https://www.nhm.ac.uk/our-science/people/jo-wilbraham.html"/>
-    <hyperlink ref="G45" r:id="rId26" display="https://orcid.org/0000-0003-4101-0611"/>
-    <hyperlink ref="E47" r:id="rId27" display="http://lattes.cnpq.br/8595257513343424"/>
-    <hyperlink ref="G47" r:id="rId28" display="https://orcid.org/0000-0002-9696-1978"/>
-    <hyperlink ref="D49" r:id="rId29" display="https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html"/>
-    <hyperlink ref="F51" r:id="rId30" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G51" r:id="rId31" display="https://orcid.org/0000-0001-8441-2106 "/>
-    <hyperlink ref="D52" r:id="rId32" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
-    <hyperlink ref="F52" r:id="rId33" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="F53" r:id="rId34" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
-    <hyperlink ref="D69" r:id="rId35" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
-    <hyperlink ref="F69" r:id="rId36" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
-    <hyperlink ref="D72" r:id="rId37" display="https://www.nhm.ac.uk/our-science/people/silvia-pressel.html"/>
-    <hyperlink ref="F72" r:id="rId38" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
-    <hyperlink ref="G72" r:id="rId39" display="https://orcid.org/0000-0001-9652-6338"/>
-    <hyperlink ref="F75" r:id="rId40" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
-    <hyperlink ref="D79" r:id="rId41" display="https://www.instagram.com/cleissa_oliveira99/"/>
-    <hyperlink ref="E79" r:id="rId42" display="http://lattes.cnpq.br/5162929358710284"/>
-    <hyperlink ref="G79" r:id="rId43" display="https://orcid.org/0009-0006-0651-3028"/>
+    <hyperlink ref="D26" r:id="rId14" display="https://www.uesc.br/centros/cme/index.php?item=conteudo_equipe.php"/>
+    <hyperlink ref="E26" r:id="rId15" display="http://lattes.cnpq.br/2078633938003826"/>
+    <hyperlink ref="F26" r:id="rId16" display="https://scholar.google.com.br/citations?user=11C9o4sAAAAJ&amp;hl=pt-PT"/>
+    <hyperlink ref="G26" r:id="rId17" display="https://orcid.org/0000-0002-1057-0432"/>
+    <hyperlink ref="E27" r:id="rId18" display="http://lattes.cnpq.br/3062370237651162"/>
+    <hyperlink ref="D28" r:id="rId19" display="https://www.instagram.com/bonesfabio/"/>
+    <hyperlink ref="E28" r:id="rId20" display="https://lattes.cnpq.br/7058195011982806"/>
+    <hyperlink ref="F28" r:id="rId21" display="https://scholar.google.com/citations?user=B_ztjnQAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G28" r:id="rId22" display="https://orcid.org/0000-0003-2956-1859"/>
+    <hyperlink ref="E33" r:id="rId23" display="http://lattes.cnpq.br/3177536756466033"/>
+    <hyperlink ref="E36" r:id="rId24" display="http://lattes.cnpq.br/4435352680317467"/>
+    <hyperlink ref="G36" r:id="rId25" display="https://orcid.org/0009-0000-5487-0915"/>
+    <hyperlink ref="E44" r:id="rId26" display="http://lattes.cnpq.br/6183123558330376"/>
+    <hyperlink ref="F44" r:id="rId27" display="https://scholar.google.com.br/citations?user=ZdlSYoAAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G44" r:id="rId28" display="https://orcid.org/0000-0002-3193-9315"/>
+    <hyperlink ref="D45" r:id="rId29" display="https://www.nhm.ac.uk/our-science/people/jo-wilbraham.html"/>
+    <hyperlink ref="G45" r:id="rId30" display="https://orcid.org/0000-0003-4101-0611"/>
+    <hyperlink ref="E47" r:id="rId31" display="http://lattes.cnpq.br/8595257513343424"/>
+    <hyperlink ref="G47" r:id="rId32" display="https://orcid.org/0000-0002-9696-1978"/>
+    <hyperlink ref="D49" r:id="rId33" display="https://www.nhm.ac.uk/our-science/people/jovita-yesilyurt.html"/>
+    <hyperlink ref="F51" r:id="rId34" display="https://scholar.google.com.br/citations?user=osGO9nEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G51" r:id="rId35" display="https://orcid.org/0000-0001-8441-2106 "/>
+    <hyperlink ref="D52" r:id="rId36" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
+    <hyperlink ref="F52" r:id="rId37" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="F53" r:id="rId38" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D69" r:id="rId39" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
+    <hyperlink ref="F69" r:id="rId40" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
+    <hyperlink ref="D72" r:id="rId41" display="https://www.nhm.ac.uk/our-science/people/silvia-pressel.html"/>
+    <hyperlink ref="F72" r:id="rId42" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
+    <hyperlink ref="G72" r:id="rId43" display="https://orcid.org/0000-0001-9652-6338"/>
+    <hyperlink ref="F75" r:id="rId44" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
+    <hyperlink ref="D79" r:id="rId45" display="https://www.instagram.com/cleissa_oliveira99/"/>
+    <hyperlink ref="E79" r:id="rId46" display="http://lattes.cnpq.br/5162929358710284"/>
+    <hyperlink ref="G79" r:id="rId47" display="https://orcid.org/0009-0006-0651-3028"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13637,6 +13668,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId44"/>
+  <drawing r:id="rId48"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update team data and rebuild team photos
</commit_message>
<xml_diff>
--- a/_input_data/tsiino_hiiwiida_team.xlsx
+++ b/_input_data/tsiino_hiiwiida_team.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="335">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -554,7 +554,7 @@
     <t xml:space="preserve">https://orcid.org/0000-0002-4871-6740</t>
   </si>
   <si>
-    <t xml:space="preserve">Gabriel Mendes Marcusso</t>
+    <t xml:space="preserve">Gabriel Marcusso</t>
   </si>
   <si>
     <t xml:space="preserve">gabrielmarcusso@hotmail.com</t>
@@ -683,7 +683,7 @@
     <t xml:space="preserve">https://orcid.org/0000-0003-2529-7691</t>
   </si>
   <si>
-    <t xml:space="preserve">Jone C R Mendes</t>
+    <t xml:space="preserve">Jone Mendes</t>
   </si>
   <si>
     <t xml:space="preserve">jonecmendes5@gmail.com</t>
@@ -779,10 +779,10 @@
     <t xml:space="preserve">Luiz Henrique Vieira Lima</t>
   </si>
   <si>
-    <t xml:space="preserve">UFRPE/PGS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://lattes.cnpq.br/8928747588815635</t>
+    <t xml:space="preserve">luizhenrique.vieira@hotmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://lattes.cnpq.br/2614964367896670</t>
   </si>
   <si>
     <t xml:space="preserve">https://orcid.org/0000-0001-7623-2826</t>
@@ -1038,7 +1038,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1160,6 +1160,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1227,7 +1242,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1304,7 +1319,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1357,7 +1388,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF0000FF"/>
+          <fgColor rgb="FF467886"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1365,7 +1396,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF467886"/>
+          <fgColor rgb="FF0000FF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2973,25 +3004,36 @@
       <c r="I57" s="12"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>251</v>
       </c>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3" t="s">
+      <c r="D58" s="19"/>
+      <c r="E58" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3" t="s">
+      <c r="F58" s="19"/>
+      <c r="G58" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="H58" s="3" t="s">
+      <c r="H58" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="I58" s="3"/>
+      <c r="I58" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="J58" s="22"/>
+      <c r="K58" s="22"/>
+      <c r="L58" s="22"/>
+      <c r="M58" s="22"/>
+      <c r="N58" s="22"/>
+      <c r="O58" s="22"/>
+      <c r="P58" s="22"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
@@ -3399,13 +3441,13 @@
         <v>10</v>
       </c>
       <c r="I77" s="3"/>
-      <c r="J77" s="19"/>
-      <c r="K77" s="19"/>
-      <c r="L77" s="19"/>
-      <c r="M77" s="19"/>
-      <c r="N77" s="19"/>
-      <c r="O77" s="19"/>
-      <c r="P77" s="19"/>
+      <c r="J77" s="23"/>
+      <c r="K77" s="23"/>
+      <c r="L77" s="23"/>
+      <c r="M77" s="23"/>
+      <c r="N77" s="23"/>
+      <c r="O77" s="23"/>
+      <c r="P77" s="23"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
@@ -3484,7 +3526,7 @@
       <c r="P80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="20" t="s">
+      <c r="A81" s="24" t="s">
         <v>330</v>
       </c>
       <c r="B81" s="3" t="s">
@@ -13714,16 +13756,18 @@
     <hyperlink ref="D55" r:id="rId39" display="https://sigaa.ufpb.br/sigaa/public/docente/portal.jsf?siape=1168469"/>
     <hyperlink ref="F55" r:id="rId40" display="https://scholar.google.com/citations?user=9P5PzkEAAAAJ&amp;hl=pt-BR"/>
     <hyperlink ref="F56" r:id="rId41" display="https://scholar.google.com/citations?user=tc_iIMkAAAAJ&amp;hl=en"/>
-    <hyperlink ref="D72" r:id="rId42" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
-    <hyperlink ref="F72" r:id="rId43" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
-    <hyperlink ref="D75" r:id="rId44" display="https://www.nhm.ac.uk/our-science/people/silvia-pressel.html"/>
-    <hyperlink ref="F75" r:id="rId45" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
-    <hyperlink ref="G75" r:id="rId46" display="https://orcid.org/0000-0001-9652-6338"/>
-    <hyperlink ref="D76" r:id="rId47" display="https://www.instagram.com/talesajr/"/>
-    <hyperlink ref="E76" r:id="rId48" display="http://lattes.cnpq.br/8055018980718354"/>
-    <hyperlink ref="F76" r:id="rId49" display="https://scholar.google.com.br/citations?user=YU7MfnAAAAAJ&amp;hl=pt-BR"/>
-    <hyperlink ref="G76" r:id="rId50" display="https://orcid.org/0000-0003-4243-9794"/>
-    <hyperlink ref="F78" r:id="rId51" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
+    <hyperlink ref="C58" r:id="rId42" display="luizhenrique.vieira@hotmail.com"/>
+    <hyperlink ref="G58" r:id="rId43" display="https://orcid.org/0000-0001-7623-2826"/>
+    <hyperlink ref="D72" r:id="rId44" display="https://www.nhm.ac.uk/our-science/people/sandra-knapp.html"/>
+    <hyperlink ref="F72" r:id="rId45" display="https://scholar.google.com/citations?user=yHApU78AAAAJ&amp;hl=en"/>
+    <hyperlink ref="D75" r:id="rId46" display="https://www.nhm.ac.uk/our-science/people/silvia-pressel.html"/>
+    <hyperlink ref="F75" r:id="rId47" display="https://scholar.google.com/citations?user=uUQ3V7UAAAAJ&amp;hl=en"/>
+    <hyperlink ref="G75" r:id="rId48" display="https://orcid.org/0000-0001-9652-6338"/>
+    <hyperlink ref="D76" r:id="rId49" display="https://www.instagram.com/talesajr/"/>
+    <hyperlink ref="E76" r:id="rId50" display="http://lattes.cnpq.br/8055018980718354"/>
+    <hyperlink ref="F76" r:id="rId51" display="https://scholar.google.com.br/citations?user=YU7MfnAAAAAJ&amp;hl=pt-BR"/>
+    <hyperlink ref="G76" r:id="rId52" display="https://orcid.org/0000-0003-4243-9794"/>
+    <hyperlink ref="F78" r:id="rId53" display="https://scholar.google.com/citations?user=na-OicAAAAAJ&amp;hl=en"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13732,6 +13776,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId52"/>
+  <drawing r:id="rId54"/>
 </worksheet>
 </file>
</xml_diff>